<commit_message>
Daily NSE scan: 2026-09-14
</commit_message>
<xml_diff>
--- a/output/2026-09-14/enriched_analysis.xlsx
+++ b/output/2026-09-14/enriched_analysis.xlsx
@@ -5873,19 +5873,19 @@
         <v>119.71</v>
       </c>
       <c r="J30" t="n">
-        <v>111.43</v>
+        <v>111.01</v>
       </c>
       <c r="K30" t="n">
-        <v>7.4</v>
+        <v>7.8</v>
       </c>
       <c r="L30" t="n">
         <v>73.48</v>
       </c>
       <c r="M30" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="N30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -5893,7 +5893,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0.207</v>
+        <v>0.198</v>
       </c>
       <c r="Q30" t="n">
         <v>227</v>
@@ -5935,10 +5935,10 @@
         <v>11.5</v>
       </c>
       <c r="AD30" t="n">
-        <v>111.7162906724512</v>
+        <v>111.3431590909091</v>
       </c>
       <c r="AE30" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="AF30" t="inlineStr">
         <is>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="AI30" t="inlineStr">
         <is>
-          <t>12-06-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
       <c r="AJ30" t="inlineStr">
@@ -5966,10 +5966,10 @@
         </is>
       </c>
       <c r="AK30" t="n">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="AL30" t="n">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="AM30" t="n">
         <v>11</v>
@@ -6827,7 +6827,7 @@
         <v>2.16</v>
       </c>
       <c r="X35" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Y35" t="b">
         <v>0</v>
@@ -11801,19 +11801,19 @@
         <v>119.71</v>
       </c>
       <c r="D30" t="n">
-        <v>111.43</v>
+        <v>111.01</v>
       </c>
       <c r="E30" t="n">
-        <v>7.4</v>
+        <v>7.8</v>
       </c>
       <c r="F30" t="n">
         <v>73.48</v>
       </c>
       <c r="G30" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="H30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>

</xml_diff>